<commit_message>
feat: adiciona gerador de dicionário de dados com IA, tipagem rápida e scraper do SENAC
- Implementa inferência rápida de tipos (CNPJ, DATE, DECIMAL) via Regex vetorizado no profiler
- Adiciona geração automática de schemas em JSON salvos junto às partições Parquet
- Cria o módulo metadata_enricher.py com integração à API do Gemini (google-genai) e cache local em DuckDB
- Adiciona o scraper de Execução Orçamentária do SENAC para todas as UFs e anos
- Adiciona suporte a variáveis de ambiente com python-dotenv
</commit_message>
<xml_diff>
--- a/outputs/sesi_relatorio_qualidade.xlsx
+++ b/outputs/sesi_relatorio_qualidade.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-09-15 16:43:44</t>
+          <t>2026-09-18 17:05:53</t>
         </is>
       </c>
     </row>

</xml_diff>